<commit_message>
Add new visit details to CSV reports
Co-authored-by: mojakimedgar <mojakimedgar@gmail.com>
</commit_message>
<xml_diff>
--- a/reports/visit_details/visit_details_gilda-katarina-mashele.xlsx
+++ b/reports/visit_details/visit_details_gilda-katarina-mashele.xlsx
@@ -419,13 +419,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:D13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="7" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="27" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -472,6 +472,248 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Gilda Katarina Mashele</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>9-Oct</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>8604030305081</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Precious Ntabiseng Molefe</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Gilda Katarina Mashele</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>9-Oct</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>9807035262087</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Piet Sebasha</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Gilda Katarina Mashele</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>9-Oct</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>0308240193083</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>euginia Makhwelepa</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Gilda Katarina Mashele</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>9-Oct</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>6704305276082</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Mandla Habile</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Gilda Katarina Mashele</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>9-Oct</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>0408050427082</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Fhulufhelo Davhana</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Gilda Katarina Mashele</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>9-Oct</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>8903251027089</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Rixongile Chabalala</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Gilda Katarina Mashele</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>9-Oct</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>9506300922082</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Kuvonakala Nkuna</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Gilda Katarina Mashele</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>9-Oct</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>0010230600081</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Gaine Chauke</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Gilda Katarina Mashele</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>9-Oct</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>0105270376087</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Kurhula Maswanganye</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Gilda Katarina Mashele</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>11-Oct</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>9801290646084</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Shongile Mayimele</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Gilda Katarina Mashele</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>11-Oct</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>9701151124082</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Damaris Mahopo</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>